<commit_message>
even more cleaning 00335756b12485f523ee5dc9861cd1d54cfd818b
</commit_message>
<xml_diff>
--- a/nr-cleaning/ig/StructureDefinition-as-dr-practitionerrole.xlsx
+++ b/nr-cleaning/ig/StructureDefinition-as-dr-practitionerrole.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2863" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="491">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-06T15:04:54+00:00</t>
+    <t>2024-03-06T15:16:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -647,13 +647,10 @@
 </t>
   </si>
   <si>
-    <t>Secteur de conventionnement du professionnel libéral auquel il a adhéré auprès de l'Assurance Maladie.</t>
+    <t>Secteur de conventionnement du professionnel libéral auquel il a adhéré auprès de l'Assurance Maladie (Synonyme : secteurConventionnement).</t>
   </si>
   <si>
     <t>Extension créée dans le cadre de l'Annuaire Santé pour décrire le secteur de conventionnement du professionnel libéral auquel il a adhéré auprès de l'Assurance Maladie.</t>
-  </si>
-  <si>
-    <t>Synonyme : secteurConventionnement</t>
   </si>
   <si>
     <t>PractitionerRole.extension:as-ext-practitionerrole-hascas</t>
@@ -3998,9 +3995,7 @@
       <c r="M19" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="N19" t="s" s="2">
-        <v>204</v>
-      </c>
+      <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
         <v>77</v>
@@ -4078,13 +4073,13 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>196</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>77</v>
@@ -4106,13 +4101,13 @@
         <v>77</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="M20" t="s" s="2">
         <v>208</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>209</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -4192,13 +4187,13 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B21" t="s" s="2">
         <v>196</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D21" t="s" s="2">
         <v>77</v>
@@ -4220,13 +4215,13 @@
         <v>77</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>213</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>214</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -4306,10 +4301,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4335,16 +4330,16 @@
         <v>111</v>
       </c>
       <c r="L22" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="M22" t="s" s="2">
         <v>216</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>217</v>
       </c>
       <c r="N22" t="s" s="2">
         <v>114</v>
       </c>
       <c r="O22" t="s" s="2">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>77</v>
@@ -4393,7 +4388,7 @@
         <v>117</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
@@ -4422,10 +4417,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4448,17 +4443,17 @@
         <v>89</v>
       </c>
       <c r="K23" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="L23" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="L23" t="s" s="2">
+      <c r="M23" t="s" s="2">
         <v>222</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>223</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" t="s" s="2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>77</v>
@@ -4495,10 +4490,10 @@
         <v>77</v>
       </c>
       <c r="AB23" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="AC23" t="s" s="2">
         <v>225</v>
-      </c>
-      <c r="AC23" t="s" s="2">
-        <v>226</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>77</v>
@@ -4507,7 +4502,7 @@
         <v>117</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4522,27 +4517,27 @@
         <v>101</v>
       </c>
       <c r="AK23" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="AL23" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AL23" t="s" s="2">
+      <c r="AM23" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="AM23" t="s" s="2">
+      <c r="AN23" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="AN23" t="s" s="2">
-        <v>230</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="B24" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="C24" t="s" s="2">
         <v>231</v>
-      </c>
-      <c r="B24" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="C24" t="s" s="2">
-        <v>232</v>
       </c>
       <c r="D24" t="s" s="2">
         <v>77</v>
@@ -4564,17 +4559,17 @@
         <v>89</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" t="s" s="2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>77</v>
@@ -4623,7 +4618,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4638,24 +4633,24 @@
         <v>101</v>
       </c>
       <c r="AK24" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="AL24" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AL24" t="s" s="2">
+      <c r="AM24" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="AM24" t="s" s="2">
+      <c r="AN24" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="AN24" t="s" s="2">
-        <v>230</v>
       </c>
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="B25" t="s" s="2">
         <v>234</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>235</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4764,10 +4759,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
+        <v>235</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>236</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>237</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4878,10 +4873,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>238</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>239</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4907,16 +4902,16 @@
         <v>173</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="M27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="N27" t="s" s="2">
+      <c r="O27" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="O27" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>77</v>
@@ -4941,31 +4936,31 @@
         <v>77</v>
       </c>
       <c r="X27" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="Y27" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="Y27" t="s" s="2">
+      <c r="Z27" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="Z27" t="s" s="2">
+      <c r="AA27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>246</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>247</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4983,7 +4978,7 @@
         <v>102</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>77</v>
@@ -4994,10 +4989,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
+        <v>248</v>
+      </c>
+      <c r="B28" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>250</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5020,19 +5015,19 @@
         <v>89</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="N28" t="s" s="2">
+      <c r="O28" t="s" s="2">
         <v>254</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>255</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>77</v>
@@ -5060,28 +5055,28 @@
         <v>153</v>
       </c>
       <c r="Y28" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="Z28" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="Z28" t="s" s="2">
+      <c r="AA28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF28" t="s" s="2">
         <v>257</v>
-      </c>
-      <c r="AA28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF28" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -5096,10 +5091,10 @@
         <v>101</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AM28" t="s" s="2">
         <v>77</v>
@@ -5110,10 +5105,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>260</v>
-      </c>
-      <c r="B29" t="s" s="2">
-        <v>261</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5139,16 +5134,16 @@
         <v>137</v>
       </c>
       <c r="L29" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="M29" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="M29" t="s" s="2">
+      <c r="N29" t="s" s="2">
         <v>263</v>
       </c>
-      <c r="N29" t="s" s="2">
+      <c r="O29" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="O29" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>77</v>
@@ -5158,46 +5153,46 @@
         <v>77</v>
       </c>
       <c r="S29" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="T29" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="T29" t="s" s="2">
+      <c r="U29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF29" t="s" s="2">
         <v>267</v>
-      </c>
-      <c r="U29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF29" t="s" s="2">
-        <v>268</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -5212,13 +5207,13 @@
         <v>101</v>
       </c>
       <c r="AK29" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="AL29" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="AL29" t="s" s="2">
+      <c r="AM29" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="AM29" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="AN29" t="s" s="2">
         <v>77</v>
@@ -5226,10 +5221,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="B30" t="s" s="2">
         <v>272</v>
-      </c>
-      <c r="B30" t="s" s="2">
-        <v>273</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5255,13 +5250,13 @@
         <v>104</v>
       </c>
       <c r="L30" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="M30" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="M30" t="s" s="2">
+      <c r="N30" t="s" s="2">
         <v>275</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>276</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -5275,43 +5270,43 @@
         <v>77</v>
       </c>
       <c r="T30" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="U30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF30" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="U30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF30" t="s" s="2">
-        <v>278</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -5326,13 +5321,13 @@
         <v>101</v>
       </c>
       <c r="AK30" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AL30" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="AL30" t="s" s="2">
+      <c r="AM30" t="s" s="2">
         <v>280</v>
-      </c>
-      <c r="AM30" t="s" s="2">
-        <v>281</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>77</v>
@@ -5340,10 +5335,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="B31" t="s" s="2">
         <v>282</v>
-      </c>
-      <c r="B31" t="s" s="2">
-        <v>283</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5366,16 +5361,16 @@
         <v>89</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="L31" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>286</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>287</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -5425,7 +5420,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5437,16 +5432,16 @@
         <v>100</v>
       </c>
       <c r="AJ31" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="AK31" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="AK31" t="s" s="2">
+      <c r="AL31" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="AL31" t="s" s="2">
+      <c r="AM31" t="s" s="2">
         <v>291</v>
-      </c>
-      <c r="AM31" t="s" s="2">
-        <v>292</v>
       </c>
       <c r="AN31" t="s" s="2">
         <v>77</v>
@@ -5454,10 +5449,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="B32" t="s" s="2">
         <v>293</v>
-      </c>
-      <c r="B32" t="s" s="2">
-        <v>294</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5480,16 +5475,16 @@
         <v>89</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="L32" t="s" s="2">
         <v>295</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="M32" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>297</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5539,7 +5534,7 @@
         <v>77</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5551,16 +5546,16 @@
         <v>100</v>
       </c>
       <c r="AJ32" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AK32" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="AK32" t="s" s="2">
+      <c r="AL32" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="AL32" t="s" s="2">
+      <c r="AM32" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="AM32" t="s" s="2">
-        <v>303</v>
       </c>
       <c r="AN32" t="s" s="2">
         <v>77</v>
@@ -5568,13 +5563,13 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="C33" t="s" s="2">
         <v>304</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>305</v>
       </c>
       <c r="D33" t="s" s="2">
         <v>77</v>
@@ -5596,17 +5591,17 @@
         <v>89</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>77</v>
@@ -5655,7 +5650,7 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5670,24 +5665,24 @@
         <v>101</v>
       </c>
       <c r="AK33" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="AL33" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AL33" t="s" s="2">
+      <c r="AM33" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="AM33" t="s" s="2">
+      <c r="AN33" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="AN33" t="s" s="2">
-        <v>230</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5796,10 +5791,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5910,10 +5905,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5939,16 +5934,16 @@
         <v>173</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="N36" t="s" s="2">
+      <c r="O36" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
@@ -5973,31 +5968,31 @@
         <v>77</v>
       </c>
       <c r="X36" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="Y36" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="Y36" t="s" s="2">
+      <c r="Z36" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="Z36" t="s" s="2">
+      <c r="AA36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF36" t="s" s="2">
         <v>246</v>
-      </c>
-      <c r="AA36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF36" t="s" s="2">
-        <v>247</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -6015,7 +6010,7 @@
         <v>102</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>77</v>
@@ -6026,10 +6021,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6052,19 +6047,19 @@
         <v>89</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="L37" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="M37" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="N37" t="s" s="2">
+      <c r="O37" t="s" s="2">
         <v>254</v>
-      </c>
-      <c r="O37" t="s" s="2">
-        <v>255</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>77</v>
@@ -6092,28 +6087,28 @@
         <v>153</v>
       </c>
       <c r="Y37" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="Z37" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="Z37" t="s" s="2">
+      <c r="AA37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF37" t="s" s="2">
         <v>257</v>
-      </c>
-      <c r="AA37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF37" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -6128,10 +6123,10 @@
         <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>77</v>
@@ -6142,10 +6137,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6171,16 +6166,16 @@
         <v>137</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="M38" t="s" s="2">
+      <c r="N38" t="s" s="2">
         <v>263</v>
       </c>
-      <c r="N38" t="s" s="2">
+      <c r="O38" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="O38" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>77</v>
@@ -6190,46 +6185,46 @@
         <v>77</v>
       </c>
       <c r="S38" t="s" s="2">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="T38" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="U38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF38" t="s" s="2">
         <v>267</v>
-      </c>
-      <c r="U38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE38" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF38" t="s" s="2">
-        <v>268</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -6244,13 +6239,13 @@
         <v>101</v>
       </c>
       <c r="AK38" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="AL38" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="AL38" t="s" s="2">
+      <c r="AM38" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="AM38" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>77</v>
@@ -6258,10 +6253,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6287,13 +6282,13 @@
         <v>104</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="N39" t="s" s="2">
         <v>275</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>276</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -6307,43 +6302,43 @@
         <v>77</v>
       </c>
       <c r="T39" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="U39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE39" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF39" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="U39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE39" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF39" t="s" s="2">
-        <v>278</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -6358,13 +6353,13 @@
         <v>101</v>
       </c>
       <c r="AK39" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AL39" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="AL39" t="s" s="2">
+      <c r="AM39" t="s" s="2">
         <v>280</v>
-      </c>
-      <c r="AM39" t="s" s="2">
-        <v>281</v>
       </c>
       <c r="AN39" t="s" s="2">
         <v>77</v>
@@ -6372,10 +6367,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6398,16 +6393,16 @@
         <v>89</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="M40" t="s" s="2">
+      <c r="N40" t="s" s="2">
         <v>286</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>287</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -6457,7 +6452,7 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6469,16 +6464,16 @@
         <v>100</v>
       </c>
       <c r="AJ40" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="AK40" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="AK40" t="s" s="2">
+      <c r="AL40" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="AL40" t="s" s="2">
+      <c r="AM40" t="s" s="2">
         <v>291</v>
-      </c>
-      <c r="AM40" t="s" s="2">
-        <v>292</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>77</v>
@@ -6486,10 +6481,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6512,16 +6507,16 @@
         <v>89</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>295</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="M41" t="s" s="2">
+      <c r="N41" t="s" s="2">
         <v>297</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -6571,7 +6566,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6583,16 +6578,16 @@
         <v>100</v>
       </c>
       <c r="AJ41" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AK41" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="AK41" t="s" s="2">
+      <c r="AL41" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="AL41" t="s" s="2">
+      <c r="AM41" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="AM41" t="s" s="2">
-        <v>303</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>77</v>
@@ -6600,10 +6595,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6626,26 +6621,26 @@
         <v>89</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="L42" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="L42" t="s" s="2">
+      <c r="M42" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="M42" t="s" s="2">
+      <c r="N42" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="N42" t="s" s="2">
+      <c r="O42" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="O42" t="s" s="2">
+      <c r="P42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q42" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="P42" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q42" t="s" s="2">
-        <v>322</v>
-      </c>
       <c r="R42" t="s" s="2">
         <v>77</v>
       </c>
@@ -6689,7 +6684,7 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6704,24 +6699,24 @@
         <v>101</v>
       </c>
       <c r="AK42" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="AL42" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="AL42" t="s" s="2">
+      <c r="AM42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN42" t="s" s="2">
         <v>324</v>
-      </c>
-      <c r="AM42" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN42" t="s" s="2">
-        <v>325</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6744,19 +6739,19 @@
         <v>89</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="M43" t="s" s="2">
+      <c r="N43" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="O43" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>329</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>77</v>
@@ -6805,7 +6800,7 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6817,27 +6812,27 @@
         <v>100</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AK43" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="AL43" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="AL43" t="s" s="2">
+      <c r="AM43" t="s" s="2">
         <v>331</v>
       </c>
-      <c r="AM43" t="s" s="2">
+      <c r="AN43" t="s" s="2">
         <v>332</v>
-      </c>
-      <c r="AN43" t="s" s="2">
-        <v>333</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6946,10 +6941,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -7060,10 +7055,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7086,16 +7081,16 @@
         <v>89</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="M46" t="s" s="2">
+      <c r="N46" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -7145,7 +7140,7 @@
         <v>77</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -7154,16 +7149,16 @@
         <v>88</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK46" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AL46" t="s" s="2">
         <v>343</v>
-      </c>
-      <c r="AL46" t="s" s="2">
-        <v>344</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>77</v>
@@ -7174,10 +7169,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7200,68 +7195,68 @@
         <v>89</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>346</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>347</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>348</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>77</v>
       </c>
       <c r="Q47" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="R47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF47" t="s" s="2">
         <v>349</v>
-      </c>
-      <c r="R47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF47" t="s" s="2">
-        <v>350</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7270,16 +7265,16 @@
         <v>88</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK47" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="AL47" t="s" s="2">
         <v>351</v>
-      </c>
-      <c r="AL47" t="s" s="2">
-        <v>352</v>
       </c>
       <c r="AM47" t="s" s="2">
         <v>77</v>
@@ -7290,10 +7285,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7316,16 +7311,16 @@
         <v>89</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>356</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>357</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -7375,7 +7370,7 @@
         <v>77</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -7387,13 +7382,13 @@
         <v>100</v>
       </c>
       <c r="AJ48" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AK48" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AM48" t="s" s="2">
         <v>77</v>
@@ -7404,10 +7399,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7430,16 +7425,16 @@
         <v>89</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="L49" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="L49" t="s" s="2">
+      <c r="M49" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="M49" t="s" s="2">
-        <v>362</v>
-      </c>
       <c r="N49" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7489,7 +7484,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7501,13 +7496,13 @@
         <v>100</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>77</v>
@@ -7518,10 +7513,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7544,19 +7539,19 @@
         <v>89</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>365</v>
       </c>
-      <c r="M50" t="s" s="2">
+      <c r="N50" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N50" t="s" s="2">
+      <c r="O50" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O50" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>77</v>
@@ -7584,16 +7579,16 @@
         <v>163</v>
       </c>
       <c r="Y50" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="Z50" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="Z50" t="s" s="2">
+      <c r="AA50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB50" t="s" s="2">
         <v>370</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>371</v>
       </c>
       <c r="AC50" s="2"/>
       <c r="AD50" t="s" s="2">
@@ -7603,7 +7598,7 @@
         <v>117</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
@@ -7618,13 +7613,13 @@
         <v>101</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL50" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM50" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN50" t="s" s="2">
         <v>77</v>
@@ -7632,13 +7627,13 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C51" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C51" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="D51" t="s" s="2">
         <v>77</v>
@@ -7660,19 +7655,19 @@
         <v>89</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="M51" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N51" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N51" t="s" s="2">
+      <c r="O51" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>77</v>
@@ -7697,11 +7692,11 @@
         <v>77</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y51" s="2"/>
       <c r="Z51" t="s" s="2">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="AA51" t="s" s="2">
         <v>77</v>
@@ -7719,7 +7714,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
@@ -7734,13 +7729,13 @@
         <v>101</v>
       </c>
       <c r="AK51" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL51" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL51" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM51" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN51" t="s" s="2">
         <v>77</v>
@@ -7748,13 +7743,13 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C52" t="s" s="2">
         <v>378</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C52" t="s" s="2">
-        <v>379</v>
       </c>
       <c r="D52" t="s" s="2">
         <v>77</v>
@@ -7776,19 +7771,19 @@
         <v>89</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="M52" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N52" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N52" t="s" s="2">
+      <c r="O52" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>77</v>
@@ -7813,11 +7808,11 @@
         <v>77</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y52" s="2"/>
       <c r="Z52" t="s" s="2">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>77</v>
@@ -7835,7 +7830,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7850,13 +7845,13 @@
         <v>101</v>
       </c>
       <c r="AK52" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL52" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL52" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM52" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>77</v>
@@ -7864,13 +7859,13 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="B53" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C53" t="s" s="2">
         <v>382</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C53" t="s" s="2">
-        <v>383</v>
       </c>
       <c r="D53" t="s" s="2">
         <v>77</v>
@@ -7892,19 +7887,19 @@
         <v>89</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="M53" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N53" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N53" t="s" s="2">
+      <c r="O53" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>77</v>
@@ -7929,11 +7924,11 @@
         <v>77</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y53" s="2"/>
       <c r="Z53" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>77</v>
@@ -7951,7 +7946,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7966,13 +7961,13 @@
         <v>101</v>
       </c>
       <c r="AK53" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL53" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL53" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM53" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN53" t="s" s="2">
         <v>77</v>
@@ -7980,13 +7975,13 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C54" t="s" s="2">
         <v>386</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C54" t="s" s="2">
-        <v>387</v>
       </c>
       <c r="D54" t="s" s="2">
         <v>77</v>
@@ -8008,19 +8003,19 @@
         <v>89</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M54" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N54" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N54" t="s" s="2">
+      <c r="O54" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O54" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>77</v>
@@ -8045,11 +8040,11 @@
         <v>77</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>77</v>
@@ -8067,7 +8062,7 @@
         <v>77</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -8082,13 +8077,13 @@
         <v>101</v>
       </c>
       <c r="AK54" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL54" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL54" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM54" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>77</v>
@@ -8096,13 +8091,13 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="B55" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C55" t="s" s="2">
         <v>390</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C55" t="s" s="2">
-        <v>391</v>
       </c>
       <c r="D55" t="s" s="2">
         <v>77</v>
@@ -8124,19 +8119,19 @@
         <v>89</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="M55" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N55" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N55" t="s" s="2">
+      <c r="O55" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O55" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>77</v>
@@ -8161,11 +8156,11 @@
         <v>77</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y55" s="2"/>
       <c r="Z55" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>77</v>
@@ -8183,7 +8178,7 @@
         <v>77</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8198,13 +8193,13 @@
         <v>101</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL55" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL55" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM55" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN55" t="s" s="2">
         <v>77</v>
@@ -8212,13 +8207,13 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C56" t="s" s="2">
         <v>394</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C56" t="s" s="2">
-        <v>395</v>
       </c>
       <c r="D56" t="s" s="2">
         <v>77</v>
@@ -8240,19 +8235,19 @@
         <v>89</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="M56" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N56" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N56" t="s" s="2">
+      <c r="O56" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>77</v>
@@ -8277,11 +8272,11 @@
         <v>77</v>
       </c>
       <c r="X56" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y56" s="2"/>
       <c r="Z56" t="s" s="2">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AA56" t="s" s="2">
         <v>77</v>
@@ -8299,7 +8294,7 @@
         <v>77</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8314,13 +8309,13 @@
         <v>101</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL56" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM56" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN56" t="s" s="2">
         <v>77</v>
@@ -8328,13 +8323,13 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="C57" t="s" s="2">
         <v>398</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C57" t="s" s="2">
-        <v>399</v>
       </c>
       <c r="D57" t="s" s="2">
         <v>77</v>
@@ -8356,19 +8351,19 @@
         <v>89</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="M57" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="N57" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="N57" t="s" s="2">
+      <c r="O57" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="O57" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>77</v>
@@ -8393,11 +8388,11 @@
         <v>77</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y57" s="2"/>
       <c r="Z57" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>77</v>
@@ -8415,7 +8410,7 @@
         <v>77</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8430,13 +8425,13 @@
         <v>101</v>
       </c>
       <c r="AK57" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AL57" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL57" t="s" s="2">
-        <v>373</v>
-      </c>
       <c r="AM57" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AN57" t="s" s="2">
         <v>77</v>
@@ -8444,10 +8439,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8470,16 +8465,16 @@
         <v>89</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>402</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>405</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -8508,11 +8503,11 @@
         <v>177</v>
       </c>
       <c r="Y58" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="Z58" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="Z58" t="s" s="2">
-        <v>407</v>
-      </c>
       <c r="AA58" t="s" s="2">
         <v>77</v>
       </c>
@@ -8529,7 +8524,7 @@
         <v>77</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
@@ -8544,13 +8539,13 @@
         <v>101</v>
       </c>
       <c r="AK58" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="AL58" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="AL58" t="s" s="2">
+      <c r="AM58" t="s" s="2">
         <v>409</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>410</v>
       </c>
       <c r="AN58" t="s" s="2">
         <v>77</v>
@@ -8558,10 +8553,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8584,16 +8579,16 @@
         <v>89</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="L59" t="s" s="2">
         <v>412</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="M59" t="s" s="2">
         <v>413</v>
       </c>
-      <c r="M59" t="s" s="2">
-        <v>414</v>
-      </c>
       <c r="N59" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -8643,7 +8638,7 @@
         <v>77</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8655,27 +8650,27 @@
         <v>100</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AK59" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL59" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="AM59" t="s" s="2">
         <v>415</v>
       </c>
-      <c r="AM59" t="s" s="2">
+      <c r="AN59" t="s" s="2">
         <v>416</v>
-      </c>
-      <c r="AN59" t="s" s="2">
-        <v>417</v>
       </c>
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8698,16 +8693,16 @@
         <v>77</v>
       </c>
       <c r="K60" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="L60" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="L60" t="s" s="2">
+      <c r="M60" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="M60" t="s" s="2">
-        <v>421</v>
-      </c>
       <c r="N60" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8757,7 +8752,7 @@
         <v>77</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>78</v>
@@ -8769,13 +8764,13 @@
         <v>100</v>
       </c>
       <c r="AJ60" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AK60" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="AL60" t="s" s="2">
         <v>422</v>
-      </c>
-      <c r="AL60" t="s" s="2">
-        <v>423</v>
       </c>
       <c r="AM60" t="s" s="2">
         <v>77</v>
@@ -8786,10 +8781,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8812,17 +8807,17 @@
         <v>89</v>
       </c>
       <c r="K61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="L61" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="L61" t="s" s="2">
+      <c r="M61" t="s" s="2">
         <v>426</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>427</v>
       </c>
       <c r="N61" s="2"/>
       <c r="O61" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>77</v>
@@ -8859,7 +8854,7 @@
         <v>77</v>
       </c>
       <c r="AB61" t="s" s="2">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AC61" s="2"/>
       <c r="AD61" t="s" s="2">
@@ -8869,7 +8864,7 @@
         <v>117</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>78</v>
@@ -8881,16 +8876,16 @@
         <v>100</v>
       </c>
       <c r="AJ61" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="AK61" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="AK61" t="s" s="2">
+      <c r="AL61" t="s" s="2">
         <v>431</v>
       </c>
-      <c r="AL61" t="s" s="2">
+      <c r="AM61" t="s" s="2">
         <v>432</v>
-      </c>
-      <c r="AM61" t="s" s="2">
-        <v>433</v>
       </c>
       <c r="AN61" t="s" s="2">
         <v>77</v>
@@ -8898,13 +8893,13 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="C62" t="s" s="2">
         <v>434</v>
-      </c>
-      <c r="B62" t="s" s="2">
-        <v>424</v>
-      </c>
-      <c r="C62" t="s" s="2">
-        <v>435</v>
       </c>
       <c r="D62" t="s" s="2">
         <v>77</v>
@@ -8926,17 +8921,17 @@
         <v>77</v>
       </c>
       <c r="K62" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="L62" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="L62" t="s" s="2">
+      <c r="M62" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>438</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="P62" t="s" s="2">
         <v>77</v>
@@ -8985,7 +8980,7 @@
         <v>77</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
@@ -8997,16 +8992,16 @@
         <v>100</v>
       </c>
       <c r="AJ62" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="AK62" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="AK62" t="s" s="2">
-        <v>431</v>
-      </c>
       <c r="AL62" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="AN62" t="s" s="2">
         <v>77</v>
@@ -9014,10 +9009,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9040,16 +9035,16 @@
         <v>77</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="L63" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="M63" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="N63" t="s" s="2">
-        <v>444</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -9099,7 +9094,7 @@
         <v>77</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>78</v>
@@ -9117,7 +9112,7 @@
         <v>77</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM63" t="s" s="2">
         <v>77</v>
@@ -9128,10 +9123,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9240,10 +9235,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9354,14 +9349,14 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" t="s" s="2">
@@ -9383,16 +9378,16 @@
         <v>111</v>
       </c>
       <c r="L66" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="M66" t="s" s="2">
         <v>450</v>
-      </c>
-      <c r="M66" t="s" s="2">
-        <v>451</v>
       </c>
       <c r="N66" t="s" s="2">
         <v>114</v>
       </c>
       <c r="O66" t="s" s="2">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P66" t="s" s="2">
         <v>77</v>
@@ -9441,7 +9436,7 @@
         <v>77</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>78</v>
@@ -9470,10 +9465,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9499,13 +9494,13 @@
         <v>173</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>455</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>456</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -9531,14 +9526,14 @@
         <v>77</v>
       </c>
       <c r="X67" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y67" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="Z67" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="Z67" t="s" s="2">
-        <v>458</v>
-      </c>
       <c r="AA67" t="s" s="2">
         <v>77</v>
       </c>
@@ -9555,7 +9550,7 @@
         <v>77</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>78</v>
@@ -9573,7 +9568,7 @@
         <v>77</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>77</v>
@@ -9584,10 +9579,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9610,13 +9605,13 @@
         <v>77</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>459</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>460</v>
-      </c>
-      <c r="M68" t="s" s="2">
-        <v>461</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -9667,7 +9662,7 @@
         <v>77</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>78</v>
@@ -9685,7 +9680,7 @@
         <v>77</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>77</v>
@@ -9696,10 +9691,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9722,16 +9717,16 @@
         <v>77</v>
       </c>
       <c r="K69" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="L69" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="L69" t="s" s="2">
+      <c r="M69" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>465</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>466</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -9781,7 +9776,7 @@
         <v>77</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>78</v>
@@ -9799,7 +9794,7 @@
         <v>77</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>77</v>
@@ -9810,10 +9805,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -9836,16 +9831,16 @@
         <v>77</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="M70" t="s" s="2">
-        <v>469</v>
-      </c>
       <c r="N70" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
@@ -9895,7 +9890,7 @@
         <v>77</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
@@ -9913,7 +9908,7 @@
         <v>77</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>77</v>
@@ -9924,10 +9919,10 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -9950,13 +9945,13 @@
         <v>77</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="L71" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="M71" t="s" s="2">
         <v>471</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>472</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -10007,7 +10002,7 @@
         <v>77</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>78</v>
@@ -10025,7 +10020,7 @@
         <v>77</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM71" t="s" s="2">
         <v>77</v>
@@ -10036,10 +10031,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10148,10 +10143,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10262,14 +10257,14 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" t="s" s="2">
@@ -10291,16 +10286,16 @@
         <v>111</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>450</v>
-      </c>
-      <c r="M74" t="s" s="2">
-        <v>451</v>
       </c>
       <c r="N74" t="s" s="2">
         <v>114</v>
       </c>
       <c r="O74" t="s" s="2">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P74" t="s" s="2">
         <v>77</v>
@@ -10349,7 +10344,7 @@
         <v>77</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>78</v>
@@ -10378,10 +10373,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10407,13 +10402,13 @@
         <v>104</v>
       </c>
       <c r="L75" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="M75" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="M75" t="s" s="2">
-        <v>478</v>
-      </c>
       <c r="N75" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -10463,7 +10458,7 @@
         <v>77</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>88</v>
@@ -10492,10 +10487,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10518,16 +10513,16 @@
         <v>77</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="M76" t="s" s="2">
-        <v>481</v>
-      </c>
       <c r="N76" t="s" s="2">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -10577,7 +10572,7 @@
         <v>77</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>78</v>
@@ -10589,13 +10584,13 @@
         <v>100</v>
       </c>
       <c r="AJ76" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AK76" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AL76" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM76" t="s" s="2">
         <v>77</v>
@@ -10606,10 +10601,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -10635,13 +10630,13 @@
         <v>104</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="M77" t="s" s="2">
-        <v>485</v>
-      </c>
       <c r="N77" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -10691,7 +10686,7 @@
         <v>77</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>78</v>
@@ -10709,7 +10704,7 @@
         <v>77</v>
       </c>
       <c r="AL77" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="AM77" t="s" s="2">
         <v>77</v>
@@ -10720,10 +10715,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -10746,19 +10741,19 @@
         <v>77</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="O78" t="s" s="2">
         <v>489</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="O78" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P78" t="s" s="2">
         <v>77</v>
@@ -10807,7 +10802,7 @@
         <v>77</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
@@ -10819,13 +10814,13 @@
         <v>100</v>
       </c>
       <c r="AJ78" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AK78" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL78" t="s" s="2">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="AM78" t="s" s="2">
         <v>77</v>

</xml_diff>